<commit_message>
Report: Pirəhmədli kəndi (via builder app, preview)
</commit_message>
<xml_diff>
--- a/cities/pirehmedli-kendi/source.xlsx
+++ b/cities/pirehmedli-kendi/source.xlsx
@@ -45,11 +45,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="4">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="[$-42C]d\ mmm\ yy;@"/>
-    <numFmt numFmtId="165" formatCode="0\ &quot;gün&quot;"/>
-    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy;@"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -428,7 +425,7 @@
         <v>projectTitle</v>
       </c>
       <c r="B2" t="str">
-        <v>PIRƏHMƏDLI KƏNDI — TIKINTI GEDIŞATI HESABATI</v>
+        <v>PIRƏHMƏDLI KƏNDI — TIKINTI GEDIŞATI HESABATI demo</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Report: Pirəhmədli kəndi (via builder app)
</commit_message>
<xml_diff>
--- a/cities/pirehmedli-kendi/source.xlsx
+++ b/cities/pirehmedli-kendi/source.xlsx
@@ -45,11 +45,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="4">
+  <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-    <numFmt numFmtId="164" formatCode="[$-42C]d\ mmm\ yy;@"/>
-    <numFmt numFmtId="165" formatCode="0\ &quot;gün&quot;"/>
-    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy;@"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -428,7 +425,7 @@
         <v>projectTitle</v>
       </c>
       <c r="B2" t="str">
-        <v>PIRƏHMƏDLI KƏNDI — TIKINTI GEDIŞATI HESABATI</v>
+        <v>PIRƏHMƏDLI KƏNDI — TIKINTI GEDIŞATI HESABATI demo</v>
       </c>
     </row>
     <row r="3">

</xml_diff>